<commit_message>
Require function-only Supabase business access and efficient RPC call contracts
</commit_message>
<xml_diff>
--- a/docs/11-management-plan/yoga-studio-management-plan.xlsx
+++ b/docs/11-management-plan/yoga-studio-management-plan.xlsx
@@ -25,6 +25,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Quality gates" sheetId="16" state="visible" r:id="rId16"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Open decisions" sheetId="17" state="visible" r:id="rId17"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Attendance acceptance" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RPC catalog" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Call budgets" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DB function gates" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Core inventory'!$A$1:$D$10</definedName>
@@ -57,10 +60,16 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="14">'Work packages'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'Quality gates'!$A$1:$F$11</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="15">'Quality gates'!$1:$1</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Open decisions'!$A$1:$E$13</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'Open decisions'!$A$1:$E$14</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="16">'Open decisions'!$1:$1</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'Attendance acceptance'!$A$1:$C$18</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="17">'Attendance acceptance'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'RPC catalog'!$A$1:$E$28</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="18">'RPC catalog'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'Call budgets'!$A$1:$C$12</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="19">'Call budgets'!$1:$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'DB function gates'!$A$1:$C$13</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="20">'DB function gates'!$1:$1</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -301,7 +310,7 @@
 </file>
 
 <file path=xl/tables/table16.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="PlanningTable16" displayName="PlanningTable16" ref="A1:E13" headerRowCount="1">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="16" name="PlanningTable16" displayName="PlanningTable16" ref="A1:E14" headerRowCount="1">
   <autoFilter ref="A1:E13"/>
   <tableColumns count="5">
     <tableColumn id="1" name="ID"/>
@@ -326,6 +335,32 @@
 </table>
 </file>
 
+<file path=xl/tables/table18.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="18" name="RpcContractCatalog" displayName="RpcContractCatalog" ref="A1:E28" headerRowCount="1">
+  <autoFilter ref="A1:E28"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Kind"/>
+    <tableColumn id="2" name="Proposed contract/operation"/>
+    <tableColumn id="3" name="Purpose / path"/>
+    <tableColumn id="4" name="Budget / returned invariant"/>
+    <tableColumn id="5" name="Implementation state"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table19.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="19" name="RpcCallBudgets" displayName="RpcCallBudgets" ref="A1:C12" headerRowCount="1">
+  <autoFilter ref="A1:C12"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Situation"/>
+    <tableColumn id="2" name="Browser business-data budget / policy"/>
+    <tableColumn id="3" name="Required safeguard"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
+</table>
+</file>
+
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="PlanningTable2" displayName="PlanningTable2" ref="A1:H13" headerRowCount="1">
   <autoFilter ref="A1:H13"/>
@@ -338,6 +373,18 @@
     <tableColumn id="6" name="Classification"/>
     <tableColumn id="7" name="Permitted readers / writers"/>
     <tableColumn id="8" name="Phase"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table20.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="20" name="DbFunctionAcceptanceGates" displayName="DbFunctionAcceptanceGates" ref="A1:C13" headerRowCount="1">
+  <autoFilter ref="A1:C13"/>
+  <tableColumns count="3">
+    <tableColumn id="1" name="Gate ID"/>
+    <tableColumn id="2" name="Required evidence"/>
+    <tableColumn id="3" name="State"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium4" showRowStripes="1"/>
 </table>
@@ -751,7 +798,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
@@ -778,7 +825,7 @@
       </c>
       <c r="B2" s="1" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-16 (updated)</t>
         </is>
       </c>
     </row>
@@ -790,7 +837,7 @@
       </c>
       <c r="B3" s="1" t="inlineStr">
         <is>
-          <t>0.2; attendance direction agreed; implementation/approval pending</t>
+          <t>0.3; function-only access and attendance direction agreed; implementation pending</t>
         </is>
       </c>
     </row>
@@ -899,6 +946,66 @@
       <c r="B12" s="1" t="inlineStr">
         <is>
           <t>Required = structural or conditionally mandatory; Phase = proposed introduction; no row is proof of implementation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="43" customHeight="1">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Business data access</t>
+        </is>
+      </c>
+      <c r="B13" s="1" t="inlineStr">
+        <is>
+          <t>All reads and writes through approved typed RPCs. api exposes functions only; app_data/private internal. Auth/Storage provider APIs are explicit exceptions.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="43" customHeight="1">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Call efficiency</t>
+        </is>
+      </c>
+      <c r="B14" s="1" t="inlineStr">
+        <is>
+          <t>One context + one screen RPC on cold navigation; one screen RPC warm. Paginate; dedupe; mutations return safe patches/counts/revisions; no per-card/per-student requests.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="43" customHeight="1">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Security execution</t>
+        </is>
+      </c>
+      <c r="B15" s="1" t="inlineStr">
+        <is>
+          <t>Invoker needs underlying grants/RLS. Definer uses owner privileges and needs reviewed ownership, least privilege and explicit checks; never assume caller RLS survives.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="43" customHeight="1">
+      <c r="A16" s="1" t="inlineStr">
+        <is>
+          <t>New specification</t>
+        </is>
+      </c>
+      <c r="B16" s="1" t="inlineStr">
+        <is>
+          <t>database-functions-and-call-policy.md — required plan direction; no live database change</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="1" t="inlineStr">
+        <is>
+          <t>Profile transition</t>
+        </is>
+      </c>
+      <c r="B17" s="1" t="inlineStr">
+        <is>
+          <t>When management tables are implemented, move business name/bio from Auth metadata to profile RPCs; avoid duplicate Auth/database writes. Email/password stay Auth API operations.</t>
         </is>
       </c>
     </row>
@@ -5383,7 +5490,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Organizations, branch membership, scoped roles and provisioning</t>
+          <t>Organizations, branch roles, RPC-only schema/grants/context and trusted provisioning</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -5398,7 +5505,7 @@
       </c>
       <c r="F3" s="3" t="inlineStr">
         <is>
-          <t>RLS isolation, role spoof, last-owner and revocation tests</t>
+          <t>RLS/anti-escalation plus DBF RPC schema/execution-mode tests</t>
         </is>
       </c>
       <c r="G3" s="3" t="inlineStr">
@@ -5420,7 +5527,7 @@
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Student/instructor/contacts, batches and enrollment</t>
+          <t>Student/instructor/contacts, batches and enrollment through typed read/write RPCs</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
@@ -5435,7 +5542,7 @@
       </c>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>Cross-tenant composite FKs; final-seat and date-interval tests</t>
+          <t>Tenant FKs; final-seat/date tests; paginated screen reads; no direct table CRUD</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
@@ -5457,7 +5564,7 @@
       </c>
       <c r="C5" s="3" t="inlineStr">
         <is>
-          <t>Dated sessions, automatic Today’s Class, instructor marking/finalization and audited corrections</t>
+          <t>Dated sessions, one-call Today’s Class/roster, RPC marking/finalization and audited corrections</t>
         </is>
       </c>
       <c r="D5" s="3" t="inlineStr">
@@ -5472,7 +5579,7 @@
       </c>
       <c r="F5" s="3" t="inlineStr">
         <is>
-          <t>ATT-01–ATT-17: server-time selection/windows, reasoned corrections, delegated Admin, cancelled/stale/offline and audit tests</t>
+          <t>ATT-01–ATT-17 plus DBF budgets: safe mutation patches, no per-student reads/refetch storms</t>
         </is>
       </c>
       <c r="G5" s="3" t="inlineStr">
@@ -5494,7 +5601,7 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Plans/subscriptions and both monthly billing policies</t>
+          <t>Plans/subscriptions, monthly billing and scoped statement RPCs</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
@@ -5509,7 +5616,7 @@
       </c>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>Golden anchor/proration/rounding/nonoverlap/idempotency cases</t>
+          <t>Golden billing cases; exact money strings, bounded statements; period/idempotency tests</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
@@ -5531,7 +5638,7 @@
       </c>
       <c r="C7" s="3" t="inlineStr">
         <is>
-          <t>Manual payments, refunds/adjustments, receipts and reports</t>
+          <t>Transactional payment/refund/receipt RPCs, scoped reports and controlled exports</t>
         </is>
       </c>
       <c r="D7" s="3" t="inlineStr">
@@ -5546,7 +5653,7 @@
       </c>
       <c r="F7" s="3" t="inlineStr">
         <is>
-          <t>No silent posted deletion; concurrency/reconciliation/scoped export tests</t>
+          <t>No silent deletion; reconciliation/audit/idempotency; aggregation/call-budget evidence</t>
         </is>
       </c>
       <c r="G7" s="3" t="inlineStr">
@@ -5568,7 +5675,7 @@
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Security/a11y/load/UAT/restore and production operations</t>
+          <t>RPC/access/security/a11y/load/UAT/restore and production operations</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
@@ -5583,7 +5690,7 @@
       </c>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>All mandatory gates, named owners and approvals</t>
+          <t>All quality gates plus DBF-01–DBF-12; query plans/call counts and approval evidence</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
@@ -5733,7 +5840,7 @@
       </c>
       <c r="C3" s="3" t="inlineStr">
         <is>
-          <t>Default-deny RLS, grants, scope, trusted roles, revocation and ordinary-user negative tests</t>
+          <t>Default-deny RLS; function-only exposed schema; least-privilege grants; invoker/definer ownership review; scoped/revoked role tests</t>
         </is>
       </c>
       <c r="D3" s="3" t="inlineStr">
@@ -5829,12 +5936,12 @@
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Pagination, indexes/plans, bounded aggregation/jobs, appropriate pooling</t>
+          <t>RPC screen-call budgets; no N+1; pagination, mutation patches, indexed plans, scoped aggregates and bounded jobs</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Agreed dataset/load report and query plans</t>
+          <t>DBF-01–DBF-12 plus measured call counts, payload sizes, workload and query-plan report</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr">
@@ -6024,7 +6131,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E13"/>
+  <dimension ref="A1:E14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
@@ -6385,8 +6492,35 @@
         </is>
       </c>
     </row>
+    <row r="14" ht="76" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>DEC-13</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Confirmed direction; implementation pending</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Supabase function-only business data access</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>All reads/writes via typed RPCs; privileged work via Edge Functions calling business RPCs; no direct table endpoints; screen-call budgets</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>User instruction, 2026-10-16; database-functions-and-call-policy.md</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E13"/>
+  <autoFilter ref="A1:E14"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
@@ -6717,6 +6851,788 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:C18"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E28"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="29" customWidth="1" min="1" max="1"/>
+    <col width="63" customWidth="1" min="2" max="2"/>
+    <col width="110" customWidth="1" min="3" max="3"/>
+    <col width="115" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Kind</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Proposed contract/operation</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Purpose / path</t>
+        </is>
+      </c>
+      <c r="D1" s="2" t="inlineStr">
+        <is>
+          <t>Budget / returned invariant</t>
+        </is>
+      </c>
+      <c r="E1" s="2" t="inlineStr">
+        <is>
+          <t>Implementation state</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>get_app_context</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Own approved profile, permitted organizations/studios/roles/capabilities and policy revision; no roster/finance preload</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>One after Auth establishes a session; reuse display context until invalidated</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>get_dashboard</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Authorized summary for one selected scope/date range; bounded today/next-session summaries and aggregate totals</t>
+        </is>
+      </c>
+      <c r="D3" s="3" t="inlineStr">
+        <is>
+          <t>One on dashboard load; no separate call per card</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>get_today_attendance</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Server time, scope, eligible session/next class or chooser, window/permission decisions, counts and first authorized roster page</t>
+        </is>
+      </c>
+      <c r="D4" s="3" t="inlineStr">
+        <is>
+          <t>One on Attendance load; selected session change is one explicit subsequent request</t>
+        </is>
+      </c>
+      <c r="E4" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>get_attendance_history</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Paginated own/authorized history with safe class/student display and correction eligibility</t>
+        </is>
+      </c>
+      <c r="D5" s="3" t="inlineStr">
+        <is>
+          <t>One per page/filter change</t>
+        </is>
+      </c>
+      <c r="E5" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>list_students</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Approved directory projection, stable cursor and page metadata</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>One per requested page, not one per student</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>get_student_detail</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>One student's safe overview plus bounded current enrollment/membership summaries; sensitive portions based on role</t>
+        </is>
+      </c>
+      <c r="D7" s="3" t="inlineStr">
+        <is>
+          <t>One for the overview; additional history pages only on demand</t>
+        </is>
+      </c>
+      <c r="E7" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>list_instructors / get_instructor_detail</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Authorized staff directory/detail; no unrelated contacts/finance</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>One per page or explicit detail load</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>list_batches / get_batch_detail</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Scoped schedule/capacity projections and bounded enrollment/session summaries</t>
+        </is>
+      </c>
+      <c r="D9" s="3" t="inlineStr">
+        <is>
+          <t>One per page or overview</t>
+        </is>
+      </c>
+      <c r="E9" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>get_student_portal</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Own upcoming classes, current attendance/membership summary and safe outstanding/payment overview</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>One initial overview; history paginated separately</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>list_memberships / get_membership_statement</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Scoped periods/dues or a bounded statement with string-serialized money and safe receipt references</t>
+        </is>
+      </c>
+      <c r="D11" s="3" t="inlineStr">
+        <is>
+          <t>One per list page/statement</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>list_payments</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Authorized scoped collection/own history page</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>One per page/filter change</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="78" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>get_settings</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Approved studio/user policy and editable-field capabilities</t>
+        </is>
+      </c>
+      <c r="D13" s="3" t="inlineStr">
+        <is>
+          <t>One when opening Settings; not every field</t>
+        </is>
+      </c>
+      <c r="E13" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="78" customHeight="1">
+      <c r="A14" s="3" t="inlineStr">
+        <is>
+          <t>Read RPC</t>
+        </is>
+      </c>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>list_audit_events</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Restricted, tenant/date/target-bounded, cursor-paginated audit projection</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>On demand only; not loaded on every page</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="78" customHeight="1">
+      <c r="A15" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Update own business profile</t>
+        </is>
+      </c>
+      <c r="C15" s="3" t="inlineStr">
+        <is>
+          <t>update_my_profile RPC</t>
+        </is>
+      </c>
+      <c r="D15" s="3" t="inlineStr">
+        <is>
+          <t>Allowlisted fields, expected version; saved safe profile returned</t>
+        </is>
+      </c>
+      <c r="E15" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="78" customHeight="1">
+      <c r="A16" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Manage student/instructor records</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Scoped create/update/archive RPCs</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>Validated fields, identity-link restrictions, expected version, minimal updated projection</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="78" customHeight="1">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B17" s="3" t="inlineStr">
+        <is>
+          <t>Change staff access / invite / ownership</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr">
+        <is>
+          <t>Authorized Edge Function + scoped database RPC + Auth Admin API when necessary</t>
+        </is>
+      </c>
+      <c r="D17" s="3" t="inlineStr">
+        <is>
+          <t>Reauthentication/MFA where required; no self-escalation; last-Owner protection; external side-effect reconciliation</t>
+        </is>
+      </c>
+      <c r="E17" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="78" customHeight="1">
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Configure studio/attendance policy</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>update_studio_policy RPC</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>Owner/delegated authority, validated policy, policy version, safe returned settings</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="78" customHeight="1">
+      <c r="A19" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B19" s="3" t="inlineStr">
+        <is>
+          <t>Create/change a batch</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>save_batch RPC</t>
+        </is>
+      </c>
+      <c r="D19" s="3" t="inlineStr">
+        <is>
+          <t>Scope, version, 60-minute rule, recurrence/conflict/capacity checks; changed summary</t>
+        </is>
+      </c>
+      <c r="E19" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="78" customHeight="1">
+      <c r="A20" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Enroll/pause/withdraw</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated enrollment RPCs</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>Locking and effective-date capacity/eligibility invariants; updated enrollment and capacity summary</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="78" customHeight="1">
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Mark/correct attendance</t>
+        </is>
+      </c>
+      <c r="C21" s="3" t="inlineStr">
+        <is>
+          <t>save_attendance_marks RPC</t>
+        </is>
+      </c>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>One deliberate save or bounded explicit batch; reasons/windows/roles/versions; changed rows, counts, server time and new revision</t>
+        </is>
+      </c>
+      <c r="E21" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="78" customHeight="1">
+      <c r="A22" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Finalize attendance</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>finalize_attendance RPC</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>Entire eligible roster/version validated; preserve Unmarked; original finalization evidence and returned summary</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="78" customHeight="1">
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>Generate sessions/periods</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>Private job entry point + transactional business functions</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Scoped idempotent generation; safe job summary, no browser job authority</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="78" customHeight="1">
+      <c r="A24" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Issue membership / change subscription</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated membership/subscription RPCs</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>Immutable issued snapshots, non-overlap, original-anchor rules, updated statement summary</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="78" customHeight="1">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Record manual receipt</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr">
+        <is>
+          <t>record_manual_payment RPC</t>
+        </is>
+      </c>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>One atomic posting, amount/currency/dues/receipt sequence/audit/idempotency checks; receipt and statement totals returned</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="78" customHeight="1">
+      <c r="A26" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Approve refund / financial adjustment</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Dedicated Owner-controlled RPC, Edge verification if external provider involved</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>Locks, remaining refundable amount, immutable linked corrections, updated statement</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="78" customHeight="1">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr">
+        <is>
+          <t>Export / receipt generation</t>
+        </is>
+      </c>
+      <c r="C27" s="3" t="inlineStr">
+        <is>
+          <t>Authorized Edge Function -&gt; business RPC -&gt; private Storage</t>
+        </is>
+      </c>
+      <c r="D27" s="3" t="inlineStr">
+        <is>
+          <t>Scope/field restrictions, bounded work/job, safe short-lived authorized delivery and audit</t>
+        </is>
+      </c>
+      <c r="E27" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="78" customHeight="1">
+      <c r="A28" s="3" t="inlineStr">
+        <is>
+          <t>Write RPC / Edge operation</t>
+        </is>
+      </c>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Future gateway callback</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Signed Edge webhook -&gt; trusted posting RPC</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>Verified event/order/account/amount/currency; durable dedupe; never browser-success authority</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr">
+        <is>
+          <t>Proposed; not created</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:E28"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">
@@ -6944,6 +7860,479 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:D10"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="40" customWidth="1" min="1" max="1"/>
+    <col width="110" customWidth="1" min="2" max="2"/>
+    <col width="115" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Situation</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Browser business-data budget / policy</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>Required safeguard</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Cold authenticated screen</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>1 context RPC + 1 requested-screen RPC</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Auth API traffic counted separately; do not preload all modules</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Warm screen / tab</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>1 bounded screen RPC</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Fetch active tab only; paginate additional requested pages</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>Today’s Class / roster</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>1 combined selection/time/permission/counts/first-page RPC</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Show complete-roster paging indicators; finalization validates all eligible students</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>Saved attendance mark/correction</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>1 RPC per deliberate save, or explicit bounded batch</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Return safe changed rows, counts, revision and server time; no whole-roster/profile refetch</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>Finalize</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>1 RPC returning summary</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Expected revision; no auto-absent, stale finalize conflicts</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>Directory search/page</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>1 per debounced filter change or requested page</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>300–500ms debounce proposed; 25 default/100 maximum page size</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Visible attendance fallback polling</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>At most one per 60s proposed while visible</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Backoff after errors; stop when hidden; writes reauthorize regardless</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>Read retry</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Up to 2 proposed automatic retries for eligible transient failures</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Bounded backoff/jitter; no automatic retry for forbidden/validation/conflict</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>Ambiguous mutation failure</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Reconcile/retry original idempotency key only</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Never create duplicate receipt/correction with new key</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>Account/branch switch</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Clear private memory/subscriptions; fetch authorized context/screen</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>No persistent private query cache or shared offline data</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>Privileged Edge workflow</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>One user action may have necessary internal RPC/provider calls</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>No claim that multiple RPCs are atomic; use one business transaction and external reconciliation</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C12"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:C13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="150" customWidth="1" min="2" max="2"/>
+    <col width="42" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="32" customHeight="1">
+      <c r="A1" s="2" t="inlineStr">
+        <is>
+          <t>Gate ID</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Required evidence</t>
+        </is>
+      </c>
+      <c r="C1" s="2" t="inlineStr">
+        <is>
+          <t>State</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="78" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>DBF-01</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Source/network tests show no application-table .from(...) CRUD or raw table REST/SQL endpoint usage; Auth SDK is an explicit exception.</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="78" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>DBF-02</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>Internal tables/schemas are not exposed by Data API, and anonymous/ordinary users cannot access them through schema/header/URL manipulation.</t>
+        </is>
+      </c>
+      <c r="C3" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="78" customHeight="1">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>DBF-03</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>Every user RPC rejects forged tenant/role/subject inputs; test suspended/revoked access and two organizations/branches.</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="78" customHeight="1">
+      <c r="A5" s="3" t="inlineStr">
+        <is>
+          <t>DBF-04</t>
+        </is>
+      </c>
+      <c r="B5" s="3" t="inlineStr">
+        <is>
+          <t>Per-function invoker/definer/owner/grants are reviewed; verify effective RLS behavior rather than assuming it.</t>
+        </is>
+      </c>
+      <c r="C5" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="78" customHeight="1">
+      <c r="A6" s="3" t="inlineStr">
+        <is>
+          <t>DBF-05</t>
+        </is>
+      </c>
+      <c r="B6" s="3" t="inlineStr">
+        <is>
+          <t>Cold dashboard/attendance uses context + one screen RPC; warm view one screen RPC; no per-card or per-student N+1 reads.</t>
+        </is>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="78" customHeight="1">
+      <c r="A7" s="3" t="inlineStr">
+        <is>
+          <t>DBF-06</t>
+        </is>
+      </c>
+      <c r="B7" s="3" t="inlineStr">
+        <is>
+          <t>Attendance save/finalize returns safe patches/counts/revisions; no whole-roster/profile refetch storm; server window checks remain authoritative.</t>
+        </is>
+      </c>
+      <c r="C7" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="78" customHeight="1">
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>DBF-07</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Pagination, bounded filters, sort/cursors and money serialization are tested with representative large datasets.</t>
+        </is>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="78" customHeight="1">
+      <c r="A9" s="3" t="inlineStr">
+        <is>
+          <t>DBF-08</t>
+        </is>
+      </c>
+      <c r="B9" s="3" t="inlineStr">
+        <is>
+          <t>Concurrency, audit atomicity, idempotency and ambiguous-network retries do not duplicate marks, enrollment, invoices, receipts or refunds.</t>
+        </is>
+      </c>
+      <c r="C9" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="78" customHeight="1">
+      <c r="A10" s="3" t="inlineStr">
+        <is>
+          <t>DBF-09</t>
+        </is>
+      </c>
+      <c r="B10" s="3" t="inlineStr">
+        <is>
+          <t>Read dedupe/backoff/foreground behavior and account/branch-switch memory isolation are tested; no private offline API cache.</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="78" customHeight="1">
+      <c r="A11" s="3" t="inlineStr">
+        <is>
+          <t>DBF-10</t>
+        </is>
+      </c>
+      <c r="B11" s="3" t="inlineStr">
+        <is>
+          <t>Query-plan/load evidence shows measured performance; a single expensive RPC is not accepted solely because its call count is low.</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="78" customHeight="1">
+      <c r="A12" s="3" t="inlineStr">
+        <is>
+          <t>DBF-11</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr">
+        <is>
+          <t>Edge Functions keep secrets server-side, authorize entry, use business RPCs and reconcile external side-effect failure; service role is not a generic read proxy.</t>
+        </is>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="78" customHeight="1">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>DBF-12</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Migration/config review confirms existing Auth/Storage/project dependencies are unaffected; implementation is verified in staging before production.</t>
+        </is>
+      </c>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>Not implemented / not executed</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A1:C13"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
   <tableParts count="1">

</xml_diff>